<commit_message>
Refactor passthrough viewer to introduce a read mode option for reading values. Implement single and multi read modes in PassthroughReader, enhancing the reading logic and error handling. Update command-line arguments to support the new read mode functionality.
</commit_message>
<xml_diff>
--- a/passthrough_map.xlsx
+++ b/passthrough_map.xlsx
@@ -43,82 +43,82 @@
     <t>DI 9 | engine</t>
   </si>
   <si>
-    <t>DI 101 | gear:P</t>
-  </si>
-  <si>
-    <t>DI 102 | gear:R</t>
-  </si>
-  <si>
-    <t>DI 103 | gear:N</t>
-  </si>
-  <si>
-    <t>DI 104 | gear:F</t>
-  </si>
-  <si>
-    <t>DI 105 | gear:H</t>
-  </si>
-  <si>
-    <t>DI 106 | gear:L</t>
-  </si>
-  <si>
-    <t>DI 107 | gear:FH</t>
-  </si>
-  <si>
-    <t>DI 111 | gear:F1</t>
-  </si>
-  <si>
-    <t>DI 112 | gear:F2</t>
-  </si>
-  <si>
-    <t>DI 113 | gear:F3</t>
-  </si>
-  <si>
-    <t>DI 114 | gear:F4</t>
-  </si>
-  <si>
-    <t>DI 115 | gear:F5</t>
-  </si>
-  <si>
-    <t>DI 116 | gear:F6</t>
-  </si>
-  <si>
-    <t>DI 117 | gear:F7</t>
-  </si>
-  <si>
-    <t>DI 118 | gear:F8</t>
-  </si>
-  <si>
-    <t>DI 119 | gear:F9</t>
-  </si>
-  <si>
-    <t>DI 121 | gear:R1</t>
-  </si>
-  <si>
-    <t>DI 122 | gear:R2</t>
-  </si>
-  <si>
-    <t>DI 130 | gear:SEL</t>
-  </si>
-  <si>
-    <t>DI 140 | gear:КПП_задний</t>
-  </si>
-  <si>
-    <t>DI 1000 | di:0</t>
-  </si>
-  <si>
-    <t>DI 1001 | di:1</t>
-  </si>
-  <si>
-    <t>DI 1002 | di:2</t>
-  </si>
-  <si>
-    <t>DI 2005 | di:5</t>
-  </si>
-  <si>
-    <t>DI 2007 | di:7</t>
-  </si>
-  <si>
-    <t>DI 2013 | di:13</t>
+    <t>DI 10 | gear:P</t>
+  </si>
+  <si>
+    <t>DI 11 | gear:R</t>
+  </si>
+  <si>
+    <t>DI 12 | gear:N</t>
+  </si>
+  <si>
+    <t>DI 13 | gear:F</t>
+  </si>
+  <si>
+    <t>DI 14 | gear:H</t>
+  </si>
+  <si>
+    <t>DI 15 | gear:L</t>
+  </si>
+  <si>
+    <t>DI 16 | gear:FH</t>
+  </si>
+  <si>
+    <t>DI 17 | gear:F1</t>
+  </si>
+  <si>
+    <t>DI 18 | gear:F2</t>
+  </si>
+  <si>
+    <t>DI 19 | gear:F3</t>
+  </si>
+  <si>
+    <t>DI 20 | gear:F4</t>
+  </si>
+  <si>
+    <t>DI 21 | gear:F5</t>
+  </si>
+  <si>
+    <t>DI 22 | gear:F6</t>
+  </si>
+  <si>
+    <t>DI 23 | gear:F7</t>
+  </si>
+  <si>
+    <t>DI 24 | gear:F8</t>
+  </si>
+  <si>
+    <t>DI 25 | gear:F9</t>
+  </si>
+  <si>
+    <t>DI 26 | gear:R1</t>
+  </si>
+  <si>
+    <t>DI 27 | gear:R2</t>
+  </si>
+  <si>
+    <t>DI 28 | gear:SEL</t>
+  </si>
+  <si>
+    <t>DI 29 | gear:КПП_задний</t>
+  </si>
+  <si>
+    <t>DI 30 | di:0</t>
+  </si>
+  <si>
+    <t>DI 31 | di:1</t>
+  </si>
+  <si>
+    <t>DI 32 | di:2</t>
+  </si>
+  <si>
+    <t>DI 33 | di:5</t>
+  </si>
+  <si>
+    <t>DI 34 | di:7</t>
+  </si>
+  <si>
+    <t>DI 35 | di:13</t>
   </si>
   <si>
     <t>Багги Segway Villain SSV</t>

</xml_diff>